<commit_message>
finalizando últimas alterações e implementando o cálculo de RMSE de cada treinamento
</commit_message>
<xml_diff>
--- a/questao-2.xlsx
+++ b/questao-2.xlsx
@@ -479,31 +479,31 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>0.2787</v>
+        <v>0.31484</v>
       </c>
       <c r="J11" t="n">
-        <v>0.46125</v>
+        <v>-0.38686</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.02204</v>
+        <v>-0.6283</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.91911</v>
+        <v>-0.23127</v>
       </c>
       <c r="M11" t="n">
-        <v>-78.7213</v>
+        <v>-78.18516</v>
       </c>
       <c r="N11" t="n">
-        <v>39.7785</v>
+        <v>39.50924</v>
       </c>
       <c r="O11" t="n">
-        <v>63.45661</v>
+        <v>63.03075</v>
       </c>
       <c r="P11" t="n">
-        <v>-18.72666</v>
+        <v>-18.59417</v>
       </c>
       <c r="Q11" t="n">
-        <v>449</v>
+        <v>423</v>
       </c>
     </row>
     <row r="12">
@@ -513,31 +513,31 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>0.01683</v>
+        <v>0.40349</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.84331</v>
+        <v>0.32486</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.11596</v>
+        <v>0.09318</v>
       </c>
       <c r="L12" t="n">
-        <v>0.94862</v>
+        <v>0.90568</v>
       </c>
       <c r="M12" t="n">
-        <v>-77.48317</v>
+        <v>-77.09650999999999</v>
       </c>
       <c r="N12" t="n">
-        <v>39.19959</v>
+        <v>39.35701</v>
       </c>
       <c r="O12" t="n">
-        <v>62.02874</v>
+        <v>61.85038</v>
       </c>
       <c r="P12" t="n">
-        <v>-18.43588</v>
+        <v>-18.38677</v>
       </c>
       <c r="Q12" t="n">
-        <v>415</v>
+        <v>407</v>
       </c>
     </row>
     <row r="13">
@@ -547,31 +547,31 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>-0.14565</v>
+        <v>-0.55462</v>
       </c>
       <c r="J13" t="n">
-        <v>0.99086</v>
+        <v>0.73414</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.3475</v>
+        <v>0.05827</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.02105</v>
+        <v>0.23956</v>
       </c>
       <c r="M13" t="n">
-        <v>-78.64565</v>
+        <v>-76.55462</v>
       </c>
       <c r="N13" t="n">
-        <v>39.25571</v>
+        <v>37.12209</v>
       </c>
       <c r="O13" t="n">
-        <v>63.10125</v>
+        <v>62.06352</v>
       </c>
       <c r="P13" t="n">
-        <v>-18.6469</v>
+        <v>-18.26844</v>
       </c>
       <c r="Q13" t="n">
-        <v>439</v>
+        <v>387</v>
       </c>
     </row>
     <row r="14">
@@ -581,31 +581,31 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>0.71505</v>
+        <v>-0.21325</v>
       </c>
       <c r="J14" t="n">
-        <v>0.07339</v>
+        <v>-0.15003</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.51551</v>
+        <v>0.97465</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.34381</v>
+        <v>-0.7234</v>
       </c>
       <c r="M14" t="n">
-        <v>-79.28494999999999</v>
+        <v>-78.21325</v>
       </c>
       <c r="N14" t="n">
-        <v>39.95804</v>
+        <v>39.38152</v>
       </c>
       <c r="O14" t="n">
-        <v>63.58569</v>
+        <v>63.0038</v>
       </c>
       <c r="P14" t="n">
-        <v>-18.82771</v>
+        <v>-18.5798</v>
       </c>
       <c r="Q14" t="n">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="15">
@@ -615,31 +615,31 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>0.06744</v>
+        <v>0.6373799999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.17863</v>
+        <v>0.02694</v>
       </c>
       <c r="K15" t="n">
-        <v>0.76244</v>
+        <v>-0.25112</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.7755</v>
+        <v>-0.83067</v>
       </c>
       <c r="M15" t="n">
-        <v>-77.93256</v>
+        <v>-78.36262000000001</v>
       </c>
       <c r="N15" t="n">
-        <v>40.23627</v>
+        <v>39.67279</v>
       </c>
       <c r="O15" t="n">
-        <v>63.01804</v>
+        <v>62.92453</v>
       </c>
       <c r="P15" t="n">
-        <v>-18.6167</v>
+        <v>-18.65132</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>445</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16">

</xml_diff>